<commit_message>
feat: implement Supabase authentication service and global AuthContext with robust profile fetching and error handling
</commit_message>
<xml_diff>
--- a/test_bulk_employees.xlsx
+++ b/test_bulk_employees.xlsx
@@ -1,41 +1,155 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\coding\osos\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A21907-4536-4B3D-B31F-7B360B67CB83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="6405" yWindow="2895" windowWidth="21600" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
+  <si>
+    <t>الاسم</t>
+  </si>
+  <si>
+    <t>الهوية الوطنية</t>
+  </si>
+  <si>
+    <t>البريد الإلكتروني</t>
+  </si>
+  <si>
+    <t>رقم الجوال</t>
+  </si>
+  <si>
+    <t>المسمى الوظيفي</t>
+  </si>
+  <si>
+    <t>المرتب</t>
+  </si>
+  <si>
+    <t>المهارات الوظيفية</t>
+  </si>
+  <si>
+    <t>اسم المستخدم</t>
+  </si>
+  <si>
+    <t>كلمة المرور</t>
+  </si>
+  <si>
+    <t>محمد أحمد العتيبي</t>
+  </si>
+  <si>
+    <t>1098765432</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>0551234567</t>
+  </si>
+  <si>
+    <t>مهندس برمجيات</t>
+  </si>
+  <si>
+    <t>البرمجة، تطوير الويب</t>
+  </si>
+  <si>
+    <t>Pass123456</t>
+  </si>
+  <si>
+    <t>عبدالله سعد الغامدي</t>
+  </si>
+  <si>
+    <t>1087654321</t>
+  </si>
+  <si>
+    <t>0559876543</t>
+  </si>
+  <si>
+    <t>محاسب</t>
+  </si>
+  <si>
+    <t>المحاسبة، Excel</t>
+  </si>
+  <si>
+    <t>خالد فهد القحطاني</t>
+  </si>
+  <si>
+    <t>1076543210</t>
+  </si>
+  <si>
+    <t>0553456789</t>
+  </si>
+  <si>
+    <t>مدير مشاريع</t>
+  </si>
+  <si>
+    <t>إدارة المشاريع، القيادة</t>
+  </si>
+  <si>
+    <t>سلطان عمر الشهري</t>
+  </si>
+  <si>
+    <t>1065432109</t>
+  </si>
+  <si>
+    <t>0554567890</t>
+  </si>
+  <si>
+    <t>فني صيانة</t>
+  </si>
+  <si>
+    <t>الصيانة الكهربائية، التكييف</t>
+  </si>
+  <si>
+    <t>ياسر حسن الدوسري</t>
+  </si>
+  <si>
+    <t>1054321098</t>
+  </si>
+  <si>
+    <t>0555678901</t>
+  </si>
+  <si>
+    <t>مسؤول موارد بشرية</t>
+  </si>
+  <si>
+    <t>إدارة الموارد البشرية، التدريب</t>
+  </si>
+  <si>
+    <t>mohammed</t>
+  </si>
+  <si>
+    <t>abdullah</t>
+  </si>
+  <si>
+    <t>khaled</t>
+  </si>
+  <si>
+    <t>sultan</t>
+  </si>
+  <si>
+    <t>yasser</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +179,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,197 +518,199 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.875" customWidth="1"/>
+    <col min="2" max="2" width="15.875" customWidth="1"/>
+    <col min="3" max="3" width="25.875" customWidth="1"/>
+    <col min="4" max="4" width="15.875" customWidth="1"/>
+    <col min="5" max="5" width="20.875" customWidth="1"/>
+    <col min="6" max="6" width="10.875" customWidth="1"/>
+    <col min="7" max="7" width="40.875" customWidth="1"/>
+    <col min="8" max="8" width="20.875" customWidth="1"/>
+    <col min="9" max="9" width="15.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>الاسم</v>
-      </c>
-      <c r="B1" t="str">
-        <v>الهوية الوطنية</v>
-      </c>
-      <c r="C1" t="str">
-        <v>البريد الإلكتروني</v>
-      </c>
-      <c r="D1" t="str">
-        <v>رقم الجوال</v>
-      </c>
-      <c r="E1" t="str">
-        <v>المسمى الوظيفي</v>
-      </c>
-      <c r="F1" t="str">
-        <v>المرتب</v>
-      </c>
-      <c r="G1" t="str">
-        <v>المهارات الوظيفية</v>
-      </c>
-      <c r="H1" t="str">
-        <v>اسم المستخدم</v>
-      </c>
-      <c r="I1" t="str">
-        <v>كلمة المرور</v>
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>محمد أحمد العتيبي</v>
-      </c>
-      <c r="B2" t="str">
-        <v>1098765432</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>0551234567</v>
-      </c>
-      <c r="E2" t="str">
-        <v>مهندس برمجيات</v>
+    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
       </c>
       <c r="F2">
         <v>8500</v>
       </c>
-      <c r="G2" t="str">
-        <v>البرمجة، تطوير الويب</v>
-      </c>
-      <c r="H2" t="str">
-        <v>mohammed.ahmed</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Pass123456</v>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>عبدالله سعد الغامدي</v>
-      </c>
-      <c r="B3" t="str">
-        <v>1087654321</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v>0559876543</v>
-      </c>
-      <c r="E3" t="str">
-        <v>محاسب</v>
+    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
       </c>
       <c r="F3">
         <v>6000</v>
       </c>
-      <c r="G3" t="str">
-        <v>المحاسبة، Excel</v>
-      </c>
-      <c r="H3" t="str">
-        <v>abdullah.saad</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Pass123456</v>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>خالد فهد القحطاني</v>
-      </c>
-      <c r="B4" t="str">
-        <v>1076543210</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>0553456789</v>
-      </c>
-      <c r="E4" t="str">
-        <v>مدير مشاريع</v>
+    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
       </c>
       <c r="F4">
         <v>12000</v>
       </c>
-      <c r="G4" t="str">
-        <v>إدارة المشاريع، القيادة</v>
-      </c>
-      <c r="H4" t="str">
-        <v>khaled.fahad</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Pass123456</v>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>سلطان عمر الشهري</v>
-      </c>
-      <c r="B5" t="str">
-        <v>1065432109</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>0554567890</v>
-      </c>
-      <c r="E5" t="str">
-        <v>فني صيانة</v>
+    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
       </c>
       <c r="F5">
         <v>5000</v>
       </c>
-      <c r="G5" t="str">
-        <v>الصيانة الكهربائية، التكييف</v>
-      </c>
-      <c r="H5" t="str">
-        <v>sultan.omar</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Pass123456</v>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>ياسر حسن الدوسري</v>
-      </c>
-      <c r="B6" t="str">
-        <v>1054321098</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>0555678901</v>
-      </c>
-      <c r="E6" t="str">
-        <v>مسؤول موارد بشرية</v>
+    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
       </c>
       <c r="F6">
         <v>7500</v>
       </c>
-      <c r="G6" t="str">
-        <v>إدارة الموارد البشرية، التدريب</v>
-      </c>
-      <c r="H6" t="str">
-        <v>yasser.hassan</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Pass123456</v>
+      <c r="G6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError sqref="A1:I1 A6:G6 A2:G2 I2 A3:G3 I3 A4:G4 I4 A5:G5 I5 I6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>